<commit_message>
OneLineRR: itemize Other Income into per-line-item columns
The Other Income section (right of Rent) was empty, so column R summed to 0.
Now each other-income line item renders as its own column (from AB) with
per-unit values, and R = SUM over them (Checking "Other Income" aggregates it).
Concessions get a dedicated column after. Falls back to a single "Other Income"
column when a source provides no per-item breakdown.

- schema: Unit.other_income_items {label: amount}
- Maven intake: records each non-Rent/non-Concession charge code (skips the
  '-' placeholder); other_income = sum of items.
- workbook: dynamic detail columns + SUM ranges.

Maven: 8 OI columns; detail totals 6,361 = source other income. Summary tabs
unchanged; Heritage regression passes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Birgo RR Exhibits - Maven @ 806v07.01.26.xlsx
+++ b/examples/outputs/Birgo RR Exhibits - Maven @ 806v07.01.26.xlsx
@@ -5971,7 +5971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:AS82"/>
+  <dimension ref="A3:AK82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.6" customWidth="1" min="1" max="1"/>
@@ -5994,6 +5994,15 @@
     <col width="12.1" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="22" max="22"/>
     <col width="12.1" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -6502,14 +6511,9 @@
           <t>Other Income</t>
         </is>
       </c>
-      <c r="AM30" s="67" t="inlineStr">
+      <c r="AK30" s="67" t="inlineStr">
         <is>
           <t>Concessions</t>
-        </is>
-      </c>
-      <c r="AS30" s="67" t="inlineStr">
-        <is>
-          <t>Employee Discounts</t>
         </is>
       </c>
     </row>
@@ -6631,22 +6635,47 @@
       </c>
       <c r="AB31" s="67" t="inlineStr">
         <is>
-          <t>Pet Fee</t>
+          <t>Building Protection Policy</t>
         </is>
       </c>
       <c r="AC31" s="67" t="inlineStr">
         <is>
-          <t>Laundry Income</t>
-        </is>
-      </c>
-      <c r="AM31" s="67" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="AS31" s="67" t="inlineStr">
-        <is>
-          <t>Employee Rent Credit</t>
+          <t>Pet Rent</t>
+        </is>
+      </c>
+      <c r="AD31" s="67" t="inlineStr">
+        <is>
+          <t>Resident Pest Control</t>
+        </is>
+      </c>
+      <c r="AE31" s="67" t="inlineStr">
+        <is>
+          <t>Resident Trash Charge</t>
+        </is>
+      </c>
+      <c r="AF31" s="67" t="inlineStr">
+        <is>
+          <t>Resident Water Charge</t>
+        </is>
+      </c>
+      <c r="AG31" s="67" t="inlineStr">
+        <is>
+          <t>WiFi/Cable Rent</t>
+        </is>
+      </c>
+      <c r="AH31" s="67" t="inlineStr">
+        <is>
+          <t>MTM Fee</t>
+        </is>
+      </c>
+      <c r="AI31" s="67" t="inlineStr">
+        <is>
+          <t>Resident Utilities (Rubs) Charge</t>
+        </is>
+      </c>
+      <c r="AK31" s="67" t="inlineStr">
+        <is>
+          <t>Concession</t>
         </is>
       </c>
     </row>
@@ -6713,19 +6742,36 @@
         <v>46474</v>
       </c>
       <c r="R32" s="81">
-        <f>SUM(AB32:AK32)</f>
+        <f>SUM(AB32:AI32)</f>
         <v/>
       </c>
       <c r="S32" s="81">
-        <f>SUM(AM32:AQ32)</f>
-        <v/>
-      </c>
-      <c r="T32" s="81">
-        <f>SUM(AS32:AW32)</f>
-        <v/>
+        <f>AK32</f>
+        <v/>
+      </c>
+      <c r="T32" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y32" s="81" t="n">
         <v>1285</v>
+      </c>
+      <c r="AB32" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC32" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD32" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE32" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF32" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG32" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="33">
@@ -6792,19 +6838,33 @@
         <v>46248</v>
       </c>
       <c r="R33" s="81">
-        <f>SUM(AB33:AK33)</f>
+        <f>SUM(AB33:AI33)</f>
         <v/>
       </c>
       <c r="S33" s="81">
-        <f>SUM(AM33:AQ33)</f>
-        <v/>
-      </c>
-      <c r="T33" s="81">
-        <f>SUM(AS33:AW33)</f>
-        <v/>
+        <f>AK33</f>
+        <v/>
+      </c>
+      <c r="T33" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y33" s="81" t="n">
         <v>1229</v>
+      </c>
+      <c r="AB33" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD33" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE33" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF33" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG33" s="81" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="34">
@@ -6871,19 +6931,33 @@
         <v>46507</v>
       </c>
       <c r="R34" s="81">
-        <f>SUM(AB34:AK34)</f>
+        <f>SUM(AB34:AI34)</f>
         <v/>
       </c>
       <c r="S34" s="81">
-        <f>SUM(AM34:AQ34)</f>
-        <v/>
-      </c>
-      <c r="T34" s="81">
-        <f>SUM(AS34:AW34)</f>
-        <v/>
+        <f>AK34</f>
+        <v/>
+      </c>
+      <c r="T34" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y34" s="81" t="n">
         <v>1249</v>
+      </c>
+      <c r="AB34" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD34" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE34" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF34" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG34" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="35">
@@ -6950,19 +7024,33 @@
         <v>46328</v>
       </c>
       <c r="R35" s="81">
-        <f>SUM(AB35:AK35)</f>
+        <f>SUM(AB35:AI35)</f>
         <v/>
       </c>
       <c r="S35" s="81">
-        <f>SUM(AM35:AQ35)</f>
-        <v/>
-      </c>
-      <c r="T35" s="81">
-        <f>SUM(AS35:AW35)</f>
-        <v/>
+        <f>AK35</f>
+        <v/>
+      </c>
+      <c r="T35" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y35" s="81" t="n">
         <v>1239</v>
+      </c>
+      <c r="AB35" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD35" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE35" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF35" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG35" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="36">
@@ -7029,19 +7117,33 @@
         <v>46507</v>
       </c>
       <c r="R36" s="81">
-        <f>SUM(AB36:AK36)</f>
+        <f>SUM(AB36:AI36)</f>
         <v/>
       </c>
       <c r="S36" s="81">
-        <f>SUM(AM36:AQ36)</f>
-        <v/>
-      </c>
-      <c r="T36" s="81">
-        <f>SUM(AS36:AW36)</f>
-        <v/>
+        <f>AK36</f>
+        <v/>
+      </c>
+      <c r="T36" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y36" s="81" t="n">
         <v>1220</v>
+      </c>
+      <c r="AB36" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD36" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE36" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF36" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG36" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="37">
@@ -7108,19 +7210,33 @@
         <v>46319</v>
       </c>
       <c r="R37" s="81">
-        <f>SUM(AB37:AK37)</f>
+        <f>SUM(AB37:AI37)</f>
         <v/>
       </c>
       <c r="S37" s="81">
-        <f>SUM(AM37:AQ37)</f>
-        <v/>
-      </c>
-      <c r="T37" s="81">
-        <f>SUM(AS37:AW37)</f>
-        <v/>
+        <f>AK37</f>
+        <v/>
+      </c>
+      <c r="T37" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y37" s="81" t="n">
         <v>1234</v>
+      </c>
+      <c r="AB37" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD37" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE37" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF37" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG37" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="38">
@@ -7178,16 +7294,15 @@
         <v/>
       </c>
       <c r="R38" s="81">
-        <f>SUM(AB38:AK38)</f>
+        <f>SUM(AB38:AI38)</f>
         <v/>
       </c>
       <c r="S38" s="81">
-        <f>SUM(AM38:AQ38)</f>
-        <v/>
-      </c>
-      <c r="T38" s="81">
-        <f>SUM(AS38:AW38)</f>
-        <v/>
+        <f>AK38</f>
+        <v/>
+      </c>
+      <c r="T38" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y38" s="81" t="n">
         <v>0</v>
@@ -7257,19 +7372,33 @@
         <v>46242</v>
       </c>
       <c r="R39" s="81">
-        <f>SUM(AB39:AK39)</f>
+        <f>SUM(AB39:AI39)</f>
         <v/>
       </c>
       <c r="S39" s="81">
-        <f>SUM(AM39:AQ39)</f>
-        <v/>
-      </c>
-      <c r="T39" s="81">
-        <f>SUM(AS39:AW39)</f>
-        <v/>
+        <f>AK39</f>
+        <v/>
+      </c>
+      <c r="T39" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y39" s="81" t="n">
         <v>1230</v>
+      </c>
+      <c r="AB39" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD39" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE39" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF39" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG39" s="81" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="40">
@@ -7336,21 +7465,35 @@
         <v>46472</v>
       </c>
       <c r="R40" s="81">
-        <f>SUM(AB40:AK40)</f>
+        <f>SUM(AB40:AI40)</f>
         <v/>
       </c>
       <c r="S40" s="81">
-        <f>SUM(AM40:AQ40)</f>
-        <v/>
-      </c>
-      <c r="T40" s="81">
-        <f>SUM(AS40:AW40)</f>
-        <v/>
+        <f>AK40</f>
+        <v/>
+      </c>
+      <c r="T40" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y40" s="81" t="n">
         <v>1249</v>
       </c>
-      <c r="AM40" s="81" t="n">
+      <c r="AB40" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD40" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE40" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF40" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG40" s="81" t="n">
+        <v>65</v>
+      </c>
+      <c r="AK40" s="81" t="n">
         <v>-374.7</v>
       </c>
     </row>
@@ -7418,19 +7561,36 @@
         <v>46244</v>
       </c>
       <c r="R41" s="81">
-        <f>SUM(AB41:AK41)</f>
+        <f>SUM(AB41:AI41)</f>
         <v/>
       </c>
       <c r="S41" s="81">
-        <f>SUM(AM41:AQ41)</f>
-        <v/>
-      </c>
-      <c r="T41" s="81">
-        <f>SUM(AS41:AW41)</f>
-        <v/>
+        <f>AK41</f>
+        <v/>
+      </c>
+      <c r="T41" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y41" s="81" t="n">
         <v>1325</v>
+      </c>
+      <c r="AB41" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC41" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD41" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE41" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF41" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG41" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="42">
@@ -7488,16 +7648,15 @@
         <v/>
       </c>
       <c r="R42" s="81">
-        <f>SUM(AB42:AK42)</f>
+        <f>SUM(AB42:AI42)</f>
         <v/>
       </c>
       <c r="S42" s="81">
-        <f>SUM(AM42:AQ42)</f>
-        <v/>
-      </c>
-      <c r="T42" s="81">
-        <f>SUM(AS42:AW42)</f>
-        <v/>
+        <f>AK42</f>
+        <v/>
+      </c>
+      <c r="T42" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y42" s="81" t="n">
         <v>0</v>
@@ -7567,19 +7726,33 @@
         <v>46396</v>
       </c>
       <c r="R43" s="81">
-        <f>SUM(AB43:AK43)</f>
+        <f>SUM(AB43:AI43)</f>
         <v/>
       </c>
       <c r="S43" s="81">
-        <f>SUM(AM43:AQ43)</f>
-        <v/>
-      </c>
-      <c r="T43" s="81">
-        <f>SUM(AS43:AW43)</f>
-        <v/>
+        <f>AK43</f>
+        <v/>
+      </c>
+      <c r="T43" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y43" s="81" t="n">
         <v>1799</v>
+      </c>
+      <c r="AB43" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD43" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE43" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF43" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG43" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="44">
@@ -7637,16 +7810,15 @@
         <v/>
       </c>
       <c r="R44" s="81">
-        <f>SUM(AB44:AK44)</f>
+        <f>SUM(AB44:AI44)</f>
         <v/>
       </c>
       <c r="S44" s="81">
-        <f>SUM(AM44:AQ44)</f>
-        <v/>
-      </c>
-      <c r="T44" s="81">
-        <f>SUM(AS44:AW44)</f>
-        <v/>
+        <f>AK44</f>
+        <v/>
+      </c>
+      <c r="T44" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y44" s="81" t="n">
         <v>0</v>
@@ -7707,16 +7879,15 @@
         <v/>
       </c>
       <c r="R45" s="81">
-        <f>SUM(AB45:AK45)</f>
+        <f>SUM(AB45:AI45)</f>
         <v/>
       </c>
       <c r="S45" s="81">
-        <f>SUM(AM45:AQ45)</f>
-        <v/>
-      </c>
-      <c r="T45" s="81">
-        <f>SUM(AS45:AW45)</f>
-        <v/>
+        <f>AK45</f>
+        <v/>
+      </c>
+      <c r="T45" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y45" s="81" t="n">
         <v>0</v>
@@ -7786,19 +7957,33 @@
         <v>46265</v>
       </c>
       <c r="R46" s="81">
-        <f>SUM(AB46:AK46)</f>
+        <f>SUM(AB46:AI46)</f>
         <v/>
       </c>
       <c r="S46" s="81">
-        <f>SUM(AM46:AQ46)</f>
-        <v/>
-      </c>
-      <c r="T46" s="81">
-        <f>SUM(AS46:AW46)</f>
-        <v/>
+        <f>AK46</f>
+        <v/>
+      </c>
+      <c r="T46" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y46" s="81" t="n">
         <v>1249</v>
+      </c>
+      <c r="AB46" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD46" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE46" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF46" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG46" s="81" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="47">
@@ -7865,19 +8050,33 @@
         <v>46280</v>
       </c>
       <c r="R47" s="81">
-        <f>SUM(AB47:AK47)</f>
+        <f>SUM(AB47:AI47)</f>
         <v/>
       </c>
       <c r="S47" s="81">
-        <f>SUM(AM47:AQ47)</f>
-        <v/>
-      </c>
-      <c r="T47" s="81">
-        <f>SUM(AS47:AW47)</f>
-        <v/>
+        <f>AK47</f>
+        <v/>
+      </c>
+      <c r="T47" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y47" s="81" t="n">
         <v>1249</v>
+      </c>
+      <c r="AB47" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD47" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE47" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF47" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG47" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="48">
@@ -7944,19 +8143,33 @@
         <v>46243</v>
       </c>
       <c r="R48" s="81">
-        <f>SUM(AB48:AK48)</f>
+        <f>SUM(AB48:AI48)</f>
         <v/>
       </c>
       <c r="S48" s="81">
-        <f>SUM(AM48:AQ48)</f>
-        <v/>
-      </c>
-      <c r="T48" s="81">
-        <f>SUM(AS48:AW48)</f>
-        <v/>
+        <f>AK48</f>
+        <v/>
+      </c>
+      <c r="T48" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y48" s="81" t="n">
         <v>1245</v>
+      </c>
+      <c r="AB48" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD48" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE48" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF48" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG48" s="81" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="49">
@@ -8023,19 +8236,36 @@
         <v>46261</v>
       </c>
       <c r="R49" s="81">
-        <f>SUM(AB49:AK49)</f>
+        <f>SUM(AB49:AI49)</f>
         <v/>
       </c>
       <c r="S49" s="81">
-        <f>SUM(AM49:AQ49)</f>
-        <v/>
-      </c>
-      <c r="T49" s="81">
-        <f>SUM(AS49:AW49)</f>
-        <v/>
+        <f>AK49</f>
+        <v/>
+      </c>
+      <c r="T49" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y49" s="81" t="n">
         <v>1215</v>
+      </c>
+      <c r="AB49" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC49" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD49" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE49" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF49" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG49" s="81" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="50">
@@ -8102,19 +8332,36 @@
         <v>46224</v>
       </c>
       <c r="R50" s="81">
-        <f>SUM(AB50:AK50)</f>
+        <f>SUM(AB50:AI50)</f>
         <v/>
       </c>
       <c r="S50" s="81">
-        <f>SUM(AM50:AQ50)</f>
-        <v/>
-      </c>
-      <c r="T50" s="81">
-        <f>SUM(AS50:AW50)</f>
-        <v/>
+        <f>AK50</f>
+        <v/>
+      </c>
+      <c r="T50" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y50" s="81" t="n">
         <v>1345</v>
+      </c>
+      <c r="AB50" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC50" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD50" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE50" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF50" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG50" s="81" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="51">
@@ -8181,19 +8428,33 @@
         <v>46438</v>
       </c>
       <c r="R51" s="81">
-        <f>SUM(AB51:AK51)</f>
+        <f>SUM(AB51:AI51)</f>
         <v/>
       </c>
       <c r="S51" s="81">
-        <f>SUM(AM51:AQ51)</f>
-        <v/>
-      </c>
-      <c r="T51" s="81">
-        <f>SUM(AS51:AW51)</f>
-        <v/>
+        <f>AK51</f>
+        <v/>
+      </c>
+      <c r="T51" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y51" s="81" t="n">
         <v>1244</v>
+      </c>
+      <c r="AB51" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD51" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE51" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF51" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG51" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="52">
@@ -8260,19 +8521,36 @@
         <v>46290</v>
       </c>
       <c r="R52" s="81">
-        <f>SUM(AB52:AK52)</f>
+        <f>SUM(AB52:AI52)</f>
         <v/>
       </c>
       <c r="S52" s="81">
-        <f>SUM(AM52:AQ52)</f>
-        <v/>
-      </c>
-      <c r="T52" s="81">
-        <f>SUM(AS52:AW52)</f>
-        <v/>
+        <f>AK52</f>
+        <v/>
+      </c>
+      <c r="T52" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y52" s="81" t="n">
         <v>1320</v>
+      </c>
+      <c r="AB52" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC52" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD52" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE52" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF52" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG52" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="53">
@@ -8339,19 +8617,33 @@
         <v>46496</v>
       </c>
       <c r="R53" s="81">
-        <f>SUM(AB53:AK53)</f>
+        <f>SUM(AB53:AI53)</f>
         <v/>
       </c>
       <c r="S53" s="81">
-        <f>SUM(AM53:AQ53)</f>
-        <v/>
-      </c>
-      <c r="T53" s="81">
-        <f>SUM(AS53:AW53)</f>
-        <v/>
+        <f>AK53</f>
+        <v/>
+      </c>
+      <c r="T53" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y53" s="81" t="n">
         <v>1049</v>
+      </c>
+      <c r="AB53" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD53" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE53" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF53" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG53" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="54">
@@ -8409,16 +8701,15 @@
         <v/>
       </c>
       <c r="R54" s="81">
-        <f>SUM(AB54:AK54)</f>
+        <f>SUM(AB54:AI54)</f>
         <v/>
       </c>
       <c r="S54" s="81">
-        <f>SUM(AM54:AQ54)</f>
-        <v/>
-      </c>
-      <c r="T54" s="81">
-        <f>SUM(AS54:AW54)</f>
-        <v/>
+        <f>AK54</f>
+        <v/>
+      </c>
+      <c r="T54" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y54" s="81" t="n">
         <v>0</v>
@@ -8479,16 +8770,15 @@
         <v/>
       </c>
       <c r="R55" s="81">
-        <f>SUM(AB55:AK55)</f>
+        <f>SUM(AB55:AI55)</f>
         <v/>
       </c>
       <c r="S55" s="81">
-        <f>SUM(AM55:AQ55)</f>
-        <v/>
-      </c>
-      <c r="T55" s="81">
-        <f>SUM(AS55:AW55)</f>
-        <v/>
+        <f>AK55</f>
+        <v/>
+      </c>
+      <c r="T55" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y55" s="81" t="n">
         <v>0</v>
@@ -8549,16 +8839,15 @@
         <v/>
       </c>
       <c r="R56" s="81">
-        <f>SUM(AB56:AK56)</f>
+        <f>SUM(AB56:AI56)</f>
         <v/>
       </c>
       <c r="S56" s="81">
-        <f>SUM(AM56:AQ56)</f>
-        <v/>
-      </c>
-      <c r="T56" s="81">
-        <f>SUM(AS56:AW56)</f>
-        <v/>
+        <f>AK56</f>
+        <v/>
+      </c>
+      <c r="T56" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y56" s="81" t="n">
         <v>0</v>
@@ -8628,19 +8917,33 @@
         <v>46227</v>
       </c>
       <c r="R57" s="81">
-        <f>SUM(AB57:AK57)</f>
+        <f>SUM(AB57:AI57)</f>
         <v/>
       </c>
       <c r="S57" s="81">
-        <f>SUM(AM57:AQ57)</f>
-        <v/>
-      </c>
-      <c r="T57" s="81">
-        <f>SUM(AS57:AW57)</f>
-        <v/>
+        <f>AK57</f>
+        <v/>
+      </c>
+      <c r="T57" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y57" s="81" t="n">
         <v>1139</v>
+      </c>
+      <c r="AB57" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD57" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE57" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF57" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG57" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="58">
@@ -8707,19 +9010,33 @@
         <v>46195</v>
       </c>
       <c r="R58" s="81">
-        <f>SUM(AB58:AK58)</f>
+        <f>SUM(AB58:AI58)</f>
         <v/>
       </c>
       <c r="S58" s="81">
-        <f>SUM(AM58:AQ58)</f>
-        <v/>
-      </c>
-      <c r="T58" s="81">
-        <f>SUM(AS58:AW58)</f>
-        <v/>
+        <f>AK58</f>
+        <v/>
+      </c>
+      <c r="T58" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y58" s="81" t="n">
         <v>1099</v>
+      </c>
+      <c r="AB58" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD58" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE58" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF58" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG58" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="59">
@@ -8783,19 +9100,36 @@
         <v>46113</v>
       </c>
       <c r="R59" s="81">
-        <f>SUM(AB59:AK59)</f>
+        <f>SUM(AB59:AI59)</f>
         <v/>
       </c>
       <c r="S59" s="81">
-        <f>SUM(AM59:AQ59)</f>
-        <v/>
-      </c>
-      <c r="T59" s="81">
-        <f>SUM(AS59:AW59)</f>
-        <v/>
+        <f>AK59</f>
+        <v/>
+      </c>
+      <c r="T59" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y59" s="81" t="n">
         <v>990</v>
+      </c>
+      <c r="AB59" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD59" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE59" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF59" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG59" s="81" t="n">
+        <v>65</v>
+      </c>
+      <c r="AH59" s="81" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="60">
@@ -8862,19 +9196,33 @@
         <v>46538</v>
       </c>
       <c r="R60" s="81">
-        <f>SUM(AB60:AK60)</f>
+        <f>SUM(AB60:AI60)</f>
         <v/>
       </c>
       <c r="S60" s="81">
-        <f>SUM(AM60:AQ60)</f>
-        <v/>
-      </c>
-      <c r="T60" s="81">
-        <f>SUM(AS60:AW60)</f>
-        <v/>
+        <f>AK60</f>
+        <v/>
+      </c>
+      <c r="T60" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y60" s="81" t="n">
         <v>1125</v>
+      </c>
+      <c r="AB60" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD60" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE60" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF60" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG60" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="61">
@@ -8941,19 +9289,33 @@
         <v>46335</v>
       </c>
       <c r="R61" s="81">
-        <f>SUM(AB61:AK61)</f>
+        <f>SUM(AB61:AI61)</f>
         <v/>
       </c>
       <c r="S61" s="81">
-        <f>SUM(AM61:AQ61)</f>
-        <v/>
-      </c>
-      <c r="T61" s="81">
-        <f>SUM(AS61:AW61)</f>
-        <v/>
+        <f>AK61</f>
+        <v/>
+      </c>
+      <c r="T61" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y61" s="81" t="n">
         <v>1179</v>
+      </c>
+      <c r="AB61" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD61" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE61" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF61" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG61" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="62">
@@ -9020,19 +9382,33 @@
         <v>46310</v>
       </c>
       <c r="R62" s="81">
-        <f>SUM(AB62:AK62)</f>
+        <f>SUM(AB62:AI62)</f>
         <v/>
       </c>
       <c r="S62" s="81">
-        <f>SUM(AM62:AQ62)</f>
-        <v/>
-      </c>
-      <c r="T62" s="81">
-        <f>SUM(AS62:AW62)</f>
-        <v/>
+        <f>AK62</f>
+        <v/>
+      </c>
+      <c r="T62" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y62" s="81" t="n">
         <v>1124</v>
+      </c>
+      <c r="AB62" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD62" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE62" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF62" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG62" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="63">
@@ -9099,19 +9475,36 @@
         <v>46381</v>
       </c>
       <c r="R63" s="81">
-        <f>SUM(AB63:AK63)</f>
+        <f>SUM(AB63:AI63)</f>
         <v/>
       </c>
       <c r="S63" s="81">
-        <f>SUM(AM63:AQ63)</f>
-        <v/>
-      </c>
-      <c r="T63" s="81">
-        <f>SUM(AS63:AW63)</f>
-        <v/>
+        <f>AK63</f>
+        <v/>
+      </c>
+      <c r="T63" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y63" s="81" t="n">
         <v>1324</v>
+      </c>
+      <c r="AB63" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC63" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD63" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE63" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF63" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG63" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="64">
@@ -9178,19 +9571,33 @@
         <v>46200</v>
       </c>
       <c r="R64" s="81">
-        <f>SUM(AB64:AK64)</f>
+        <f>SUM(AB64:AI64)</f>
         <v/>
       </c>
       <c r="S64" s="81">
-        <f>SUM(AM64:AQ64)</f>
-        <v/>
-      </c>
-      <c r="T64" s="81">
-        <f>SUM(AS64:AW64)</f>
-        <v/>
+        <f>AK64</f>
+        <v/>
+      </c>
+      <c r="T64" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y64" s="81" t="n">
         <v>1114</v>
+      </c>
+      <c r="AB64" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD64" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE64" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF64" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG64" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="65">
@@ -9257,19 +9664,33 @@
         <v>46352</v>
       </c>
       <c r="R65" s="81">
-        <f>SUM(AB65:AK65)</f>
+        <f>SUM(AB65:AI65)</f>
         <v/>
       </c>
       <c r="S65" s="81">
-        <f>SUM(AM65:AQ65)</f>
-        <v/>
-      </c>
-      <c r="T65" s="81">
-        <f>SUM(AS65:AW65)</f>
-        <v/>
+        <f>AK65</f>
+        <v/>
+      </c>
+      <c r="T65" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y65" s="81" t="n">
         <v>1245</v>
+      </c>
+      <c r="AB65" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD65" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE65" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF65" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG65" s="81" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="66">
@@ -9336,19 +9757,33 @@
         <v>46493</v>
       </c>
       <c r="R66" s="81">
-        <f>SUM(AB66:AK66)</f>
+        <f>SUM(AB66:AI66)</f>
         <v/>
       </c>
       <c r="S66" s="81">
-        <f>SUM(AM66:AQ66)</f>
-        <v/>
-      </c>
-      <c r="T66" s="81">
-        <f>SUM(AS66:AW66)</f>
-        <v/>
+        <f>AK66</f>
+        <v/>
+      </c>
+      <c r="T66" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y66" s="81" t="n">
         <v>1059</v>
+      </c>
+      <c r="AB66" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD66" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE66" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF66" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG66" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="67">
@@ -9415,19 +9850,33 @@
         <v>46354</v>
       </c>
       <c r="R67" s="81">
-        <f>SUM(AB67:AK67)</f>
+        <f>SUM(AB67:AI67)</f>
         <v/>
       </c>
       <c r="S67" s="81">
-        <f>SUM(AM67:AQ67)</f>
-        <v/>
-      </c>
-      <c r="T67" s="81">
-        <f>SUM(AS67:AW67)</f>
-        <v/>
+        <f>AK67</f>
+        <v/>
+      </c>
+      <c r="T67" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y67" s="81" t="n">
         <v>1384</v>
+      </c>
+      <c r="AB67" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD67" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE67" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF67" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG67" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="68">
@@ -9485,16 +9934,15 @@
         <v/>
       </c>
       <c r="R68" s="81">
-        <f>SUM(AB68:AK68)</f>
+        <f>SUM(AB68:AI68)</f>
         <v/>
       </c>
       <c r="S68" s="81">
-        <f>SUM(AM68:AQ68)</f>
-        <v/>
-      </c>
-      <c r="T68" s="81">
-        <f>SUM(AS68:AW68)</f>
-        <v/>
+        <f>AK68</f>
+        <v/>
+      </c>
+      <c r="T68" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y68" s="81" t="n">
         <v>0</v>
@@ -9564,19 +10012,36 @@
         <v>46446</v>
       </c>
       <c r="R69" s="81">
-        <f>SUM(AB69:AK69)</f>
+        <f>SUM(AB69:AI69)</f>
         <v/>
       </c>
       <c r="S69" s="81">
-        <f>SUM(AM69:AQ69)</f>
-        <v/>
-      </c>
-      <c r="T69" s="81">
-        <f>SUM(AS69:AW69)</f>
-        <v/>
+        <f>AK69</f>
+        <v/>
+      </c>
+      <c r="T69" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y69" s="81" t="n">
         <v>1184</v>
+      </c>
+      <c r="AB69" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC69" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD69" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE69" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF69" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG69" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="70">
@@ -9643,19 +10108,33 @@
         <v>46403</v>
       </c>
       <c r="R70" s="81">
-        <f>SUM(AB70:AK70)</f>
+        <f>SUM(AB70:AI70)</f>
         <v/>
       </c>
       <c r="S70" s="81">
-        <f>SUM(AM70:AQ70)</f>
-        <v/>
-      </c>
-      <c r="T70" s="81">
-        <f>SUM(AS70:AW70)</f>
-        <v/>
+        <f>AK70</f>
+        <v/>
+      </c>
+      <c r="T70" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y70" s="81" t="n">
         <v>1255</v>
+      </c>
+      <c r="AB70" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD70" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE70" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF70" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG70" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="71">
@@ -9722,19 +10201,33 @@
         <v>46233</v>
       </c>
       <c r="R71" s="81">
-        <f>SUM(AB71:AK71)</f>
+        <f>SUM(AB71:AI71)</f>
         <v/>
       </c>
       <c r="S71" s="81">
-        <f>SUM(AM71:AQ71)</f>
-        <v/>
-      </c>
-      <c r="T71" s="81">
-        <f>SUM(AS71:AW71)</f>
-        <v/>
+        <f>AK71</f>
+        <v/>
+      </c>
+      <c r="T71" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y71" s="81" t="n">
         <v>1149</v>
+      </c>
+      <c r="AB71" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD71" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE71" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF71" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG71" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="72">
@@ -9792,16 +10285,15 @@
         <v/>
       </c>
       <c r="R72" s="81">
-        <f>SUM(AB72:AK72)</f>
+        <f>SUM(AB72:AI72)</f>
         <v/>
       </c>
       <c r="S72" s="81">
-        <f>SUM(AM72:AQ72)</f>
-        <v/>
-      </c>
-      <c r="T72" s="81">
-        <f>SUM(AS72:AW72)</f>
-        <v/>
+        <f>AK72</f>
+        <v/>
+      </c>
+      <c r="T72" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y72" s="81" t="n">
         <v>0</v>
@@ -9871,19 +10363,33 @@
         <v>46215</v>
       </c>
       <c r="R73" s="81">
-        <f>SUM(AB73:AK73)</f>
+        <f>SUM(AB73:AI73)</f>
         <v/>
       </c>
       <c r="S73" s="81">
-        <f>SUM(AM73:AQ73)</f>
-        <v/>
-      </c>
-      <c r="T73" s="81">
-        <f>SUM(AS73:AW73)</f>
-        <v/>
+        <f>AK73</f>
+        <v/>
+      </c>
+      <c r="T73" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y73" s="81" t="n">
         <v>1330</v>
+      </c>
+      <c r="AB73" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD73" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE73" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF73" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG73" s="81" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="74">
@@ -9950,19 +10456,36 @@
         <v>46172</v>
       </c>
       <c r="R74" s="81">
-        <f>SUM(AB74:AK74)</f>
+        <f>SUM(AB74:AI74)</f>
         <v/>
       </c>
       <c r="S74" s="81">
-        <f>SUM(AM74:AQ74)</f>
-        <v/>
-      </c>
-      <c r="T74" s="81">
-        <f>SUM(AS74:AW74)</f>
-        <v/>
+        <f>AK74</f>
+        <v/>
+      </c>
+      <c r="T74" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y74" s="81" t="n">
         <v>1185</v>
+      </c>
+      <c r="AB74" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC74" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD74" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE74" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF74" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG74" s="81" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="75">
@@ -10029,19 +10552,36 @@
         <v>46503</v>
       </c>
       <c r="R75" s="81">
-        <f>SUM(AB75:AK75)</f>
+        <f>SUM(AB75:AI75)</f>
         <v/>
       </c>
       <c r="S75" s="81">
-        <f>SUM(AM75:AQ75)</f>
-        <v/>
-      </c>
-      <c r="T75" s="81">
-        <f>SUM(AS75:AW75)</f>
-        <v/>
+        <f>AK75</f>
+        <v/>
+      </c>
+      <c r="T75" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y75" s="81" t="n">
         <v>1355</v>
+      </c>
+      <c r="AB75" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC75" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AD75" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE75" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF75" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG75" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="76">
@@ -10108,19 +10648,33 @@
         <v>46262</v>
       </c>
       <c r="R76" s="81">
-        <f>SUM(AB76:AK76)</f>
+        <f>SUM(AB76:AI76)</f>
         <v/>
       </c>
       <c r="S76" s="81">
-        <f>SUM(AM76:AQ76)</f>
-        <v/>
-      </c>
-      <c r="T76" s="81">
-        <f>SUM(AS76:AW76)</f>
-        <v/>
+        <f>AK76</f>
+        <v/>
+      </c>
+      <c r="T76" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y76" s="81" t="n">
         <v>1334</v>
+      </c>
+      <c r="AB76" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD76" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE76" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF76" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG76" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="77">
@@ -10187,19 +10741,33 @@
         <v>46186</v>
       </c>
       <c r="R77" s="81">
-        <f>SUM(AB77:AK77)</f>
+        <f>SUM(AB77:AI77)</f>
         <v/>
       </c>
       <c r="S77" s="81">
-        <f>SUM(AM77:AQ77)</f>
-        <v/>
-      </c>
-      <c r="T77" s="81">
-        <f>SUM(AS77:AW77)</f>
-        <v/>
+        <f>AK77</f>
+        <v/>
+      </c>
+      <c r="T77" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y77" s="81" t="n">
         <v>1124</v>
+      </c>
+      <c r="AB77" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD77" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE77" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF77" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG77" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="78">
@@ -10266,19 +10834,33 @@
         <v>46219</v>
       </c>
       <c r="R78" s="81">
-        <f>SUM(AB78:AK78)</f>
+        <f>SUM(AB78:AI78)</f>
         <v/>
       </c>
       <c r="S78" s="81">
-        <f>SUM(AM78:AQ78)</f>
-        <v/>
-      </c>
-      <c r="T78" s="81">
-        <f>SUM(AS78:AW78)</f>
-        <v/>
+        <f>AK78</f>
+        <v/>
+      </c>
+      <c r="T78" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y78" s="81" t="n">
         <v>1334</v>
+      </c>
+      <c r="AB78" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD78" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE78" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF78" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG78" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="79">
@@ -10345,19 +10927,33 @@
         <v>46476</v>
       </c>
       <c r="R79" s="81">
-        <f>SUM(AB79:AK79)</f>
+        <f>SUM(AB79:AI79)</f>
         <v/>
       </c>
       <c r="S79" s="81">
-        <f>SUM(AM79:AQ79)</f>
-        <v/>
-      </c>
-      <c r="T79" s="81">
-        <f>SUM(AS79:AW79)</f>
-        <v/>
+        <f>AK79</f>
+        <v/>
+      </c>
+      <c r="T79" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y79" s="81" t="n">
         <v>1394</v>
+      </c>
+      <c r="AB79" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD79" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE79" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF79" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG79" s="81" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="80">
@@ -10424,19 +11020,36 @@
         <v>46416</v>
       </c>
       <c r="R80" s="81">
-        <f>SUM(AB80:AK80)</f>
+        <f>SUM(AB80:AI80)</f>
         <v/>
       </c>
       <c r="S80" s="81">
-        <f>SUM(AM80:AQ80)</f>
-        <v/>
-      </c>
-      <c r="T80" s="81">
-        <f>SUM(AS80:AW80)</f>
-        <v/>
+        <f>AK80</f>
+        <v/>
+      </c>
+      <c r="T80" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y80" s="81" t="n">
         <v>1300</v>
+      </c>
+      <c r="AB80" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD80" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE80" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF80" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG80" s="81" t="n">
+        <v>65</v>
+      </c>
+      <c r="AI80" s="81" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="81">
@@ -10503,19 +11116,39 @@
         <v>46185</v>
       </c>
       <c r="R81" s="81">
-        <f>SUM(AB81:AK81)</f>
+        <f>SUM(AB81:AI81)</f>
         <v/>
       </c>
       <c r="S81" s="81">
-        <f>SUM(AM81:AQ81)</f>
-        <v/>
-      </c>
-      <c r="T81" s="81">
-        <f>SUM(AS81:AW81)</f>
-        <v/>
+        <f>AK81</f>
+        <v/>
+      </c>
+      <c r="T81" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y81" s="81" t="n">
         <v>1145</v>
+      </c>
+      <c r="AB81" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC81" s="81" t="n">
+        <v>65</v>
+      </c>
+      <c r="AD81" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE81" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF81" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG81" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI81" s="81" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="82">
@@ -10582,19 +11215,36 @@
         <v>46232</v>
       </c>
       <c r="R82" s="81">
-        <f>SUM(AB82:AK82)</f>
+        <f>SUM(AB82:AI82)</f>
         <v/>
       </c>
       <c r="S82" s="81">
-        <f>SUM(AM82:AQ82)</f>
-        <v/>
-      </c>
-      <c r="T82" s="81">
-        <f>SUM(AS82:AW82)</f>
-        <v/>
+        <f>AK82</f>
+        <v/>
+      </c>
+      <c r="T82" s="81" t="n">
+        <v>0</v>
       </c>
       <c r="Y82" s="81" t="n">
         <v>1189</v>
+      </c>
+      <c r="AB82" s="81" t="n">
+        <v>15</v>
+      </c>
+      <c r="AD82" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE82" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF82" s="81" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG82" s="81" t="n">
+        <v>65</v>
+      </c>
+      <c r="AI82" s="81" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Populate Move Out on the OneLineRR tab
The OneLineRR "Move Out" column (Q) was never filled because Unit had no
move_out field. Added Unit.move_out (with date coercion), mapped it in the
intakes (Maven "Expected Move-Out"; Station J Town "Move Out"), and the
OneLineRR writes Q when available.

Maven: 3 move-outs (the notice units). Heritage regression passes. Docs updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Birgo RR Exhibits - Maven @ 806v07.01.26.xlsx
+++ b/examples/outputs/Birgo RR Exhibits - Maven @ 806v07.01.26.xlsx
@@ -6849,6 +6849,9 @@
       <c r="P33" s="82" t="n">
         <v>46248</v>
       </c>
+      <c r="Q33" s="82" t="n">
+        <v>46295</v>
+      </c>
       <c r="R33" s="81">
         <f>SUM(AB33:AI33)</f>
         <v/>
@@ -7403,6 +7406,9 @@
       <c r="P39" s="82" t="n">
         <v>46242</v>
       </c>
+      <c r="Q39" s="82" t="n">
+        <v>46295</v>
+      </c>
       <c r="R39" s="81">
         <f>SUM(AB39:AI39)</f>
         <v/>
@@ -8423,6 +8429,9 @@
       <c r="P50" s="82" t="n">
         <v>46224</v>
       </c>
+      <c r="Q50" s="82" t="n">
+        <v>46204</v>
+      </c>
       <c r="R50" s="81">
         <f>SUM(AB50:AI50)</f>
         <v/>

</xml_diff>

<commit_message>
Route employee-discount charges to the Employee Discount section
Any charge whose name contains "employee discount" is now classified to the
employee-discount field instead of concession. Pres. RR shows it in col X; the
OneLineRR renders an "Employee Discounts" detail column with T = SUM. Not
netted into in-place rent (netting stays concession-only).

Maven: "Concession-Employee Rent Discount Special" (-374.70) on 800-2C moves
concession -> employee discount. Grand scheduled total unchanged (58,021.30).
Heritage regression passes. Docs + iteration log (#23) updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Birgo RR Exhibits - Maven @ 806v07.01.26.xlsx
+++ b/examples/outputs/Birgo RR Exhibits - Maven @ 806v07.01.26.xlsx
@@ -915,13 +915,13 @@
         <v>1.80252000477726</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>29100.3</v>
+        <v>29475</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>1164.012</v>
+        <v>1179</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>1.815818045675777</v>
+        <v>1.839198801946836</v>
       </c>
       <c r="P6" s="11" t="n">
         <v>1325</v>
@@ -1065,13 +1065,13 @@
         <v>1.725271002710027</v>
       </c>
       <c r="M9" s="17" t="n">
-        <v>51660.3</v>
+        <v>52035</v>
       </c>
       <c r="N9" s="17" t="n">
-        <v>1230.007142857143</v>
+        <v>1238.928571428571</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>1.700414732892268</v>
+        <v>1.712748099140911</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>1398.529411764706</v>
@@ -1184,7 +1184,7 @@
       <c r="E19" s="20" t="n"/>
       <c r="F19" s="20" t="n"/>
       <c r="G19" s="24" t="n">
-        <v>619923.6000000001</v>
+        <v>624420</v>
       </c>
     </row>
     <row r="20">
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="W49" s="27" t="n">
-        <v>51660.3</v>
+        <v>52035</v>
       </c>
     </row>
     <row r="50">
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="W50" s="27" t="n">
-        <v>-374.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1555,31 +1555,31 @@
         <v>1167.8</v>
       </c>
       <c r="L7" s="11" t="n">
-        <v>1164.012</v>
+        <v>1179</v>
       </c>
       <c r="M7" s="39" t="n">
-        <v>0.9967562938859393</v>
+        <v>1.009590683336188</v>
       </c>
       <c r="N7" s="38" t="n">
-        <v>1133.53</v>
+        <v>1171</v>
       </c>
       <c r="O7" s="40" t="n">
         <v>10</v>
       </c>
       <c r="P7" s="11" t="n">
-        <v>1121.144444444444</v>
+        <v>1162.777777777778</v>
       </c>
       <c r="Q7" s="40" t="n">
         <v>9</v>
       </c>
       <c r="R7" s="11" t="n">
-        <v>1140.328571428571</v>
+        <v>1193.857142857143</v>
       </c>
       <c r="S7" s="40" t="n">
         <v>7</v>
       </c>
       <c r="T7" s="11" t="n">
-        <v>1142.883333333333</v>
+        <v>1205.333333333333</v>
       </c>
       <c r="U7" s="40" t="n">
         <v>6</v>
@@ -1758,10 +1758,10 @@
         <v>1252.452380952381</v>
       </c>
       <c r="L10" s="17" t="n">
-        <v>1230.007142857143</v>
+        <v>1238.928571428571</v>
       </c>
       <c r="M10" s="43" t="n">
-        <v>0.9820789688801019</v>
+        <v>0.9892021367602607</v>
       </c>
       <c r="N10" s="42" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="AB66" s="27" t="n">
-        <v>51660.3</v>
+        <v>52035</v>
       </c>
     </row>
   </sheetData>
@@ -2063,13 +2063,13 @@
         <v>1.80252000477726</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>29100.3</v>
+        <v>29475</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>1164.012</v>
+        <v>1179</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>1.815818045675777</v>
+        <v>1.839198801946836</v>
       </c>
       <c r="P6" s="11" t="n">
         <v>1325</v>
@@ -2160,13 +2160,13 @@
         <v>1.725271002710027</v>
       </c>
       <c r="M8" s="17" t="n">
-        <v>51660.3</v>
+        <v>52035</v>
       </c>
       <c r="N8" s="17" t="n">
-        <v>1230.007142857143</v>
+        <v>1238.928571428571</v>
       </c>
       <c r="O8" s="18" t="n">
-        <v>1.700414732892268</v>
+        <v>1.712748099140911</v>
       </c>
       <c r="P8" s="17" t="inlineStr">
         <is>
@@ -2281,7 +2281,7 @@
       <c r="E18" s="20" t="n"/>
       <c r="F18" s="20" t="n"/>
       <c r="G18" s="24" t="n">
-        <v>619923.6000000001</v>
+        <v>624420</v>
       </c>
     </row>
     <row r="19">
@@ -3244,10 +3244,10 @@
         <v>1249</v>
       </c>
       <c r="W16" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="58" t="n">
         <v>-374.7</v>
-      </c>
-      <c r="X16" s="58" t="n">
-        <v>0</v>
       </c>
       <c r="Y16" s="58" t="n">
         <v>134</v>
@@ -5948,13 +5948,13 @@
         <v>66209</v>
       </c>
       <c r="V59" s="64" t="n">
-        <v>51660.3</v>
+        <v>52035</v>
       </c>
       <c r="W59" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="X59" s="64" t="n">
         <v>-374.7</v>
-      </c>
-      <c r="X59" s="64" t="n">
-        <v>0</v>
       </c>
       <c r="Y59" s="64" t="n">
         <v>6361</v>
@@ -5983,7 +5983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:AK82"/>
+  <dimension ref="A3:AM82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.6" customWidth="1" min="1" max="1"/>
@@ -6014,7 +6014,7 @@
     <col width="13" customWidth="1" min="33" max="33"/>
     <col width="13" customWidth="1" min="34" max="34"/>
     <col width="13" customWidth="1" min="35" max="35"/>
-    <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -6523,9 +6523,9 @@
           <t>Other Income</t>
         </is>
       </c>
-      <c r="AK30" s="67" t="inlineStr">
-        <is>
-          <t>Concessions</t>
+      <c r="AM30" s="67" t="inlineStr">
+        <is>
+          <t>Employee Discounts</t>
         </is>
       </c>
     </row>
@@ -6685,9 +6685,9 @@
           <t>Resident Utilities (Rubs) Charge</t>
         </is>
       </c>
-      <c r="AK31" s="67" t="inlineStr">
-        <is>
-          <t>Concession</t>
+      <c r="AM31" s="67" t="inlineStr">
+        <is>
+          <t>Employee Discount</t>
         </is>
       </c>
     </row>
@@ -6757,12 +6757,12 @@
         <f>SUM(AB32:AI32)</f>
         <v/>
       </c>
-      <c r="S32" s="81">
-        <f>AK32</f>
-        <v/>
-      </c>
-      <c r="T32" s="81" t="n">
-        <v>0</v>
+      <c r="S32" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" s="81">
+        <f>AM32</f>
+        <v/>
       </c>
       <c r="Y32" s="81" t="n">
         <v>1285</v>
@@ -6856,12 +6856,12 @@
         <f>SUM(AB33:AI33)</f>
         <v/>
       </c>
-      <c r="S33" s="81">
-        <f>AK33</f>
-        <v/>
-      </c>
-      <c r="T33" s="81" t="n">
-        <v>0</v>
+      <c r="S33" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" s="81">
+        <f>AM33</f>
+        <v/>
       </c>
       <c r="Y33" s="81" t="n">
         <v>1229</v>
@@ -6949,12 +6949,12 @@
         <f>SUM(AB34:AI34)</f>
         <v/>
       </c>
-      <c r="S34" s="81">
-        <f>AK34</f>
-        <v/>
-      </c>
-      <c r="T34" s="81" t="n">
-        <v>0</v>
+      <c r="S34" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="81">
+        <f>AM34</f>
+        <v/>
       </c>
       <c r="Y34" s="81" t="n">
         <v>1249</v>
@@ -7042,12 +7042,12 @@
         <f>SUM(AB35:AI35)</f>
         <v/>
       </c>
-      <c r="S35" s="81">
-        <f>AK35</f>
-        <v/>
-      </c>
-      <c r="T35" s="81" t="n">
-        <v>0</v>
+      <c r="S35" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="81">
+        <f>AM35</f>
+        <v/>
       </c>
       <c r="Y35" s="81" t="n">
         <v>1239</v>
@@ -7135,12 +7135,12 @@
         <f>SUM(AB36:AI36)</f>
         <v/>
       </c>
-      <c r="S36" s="81">
-        <f>AK36</f>
-        <v/>
-      </c>
-      <c r="T36" s="81" t="n">
-        <v>0</v>
+      <c r="S36" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" s="81">
+        <f>AM36</f>
+        <v/>
       </c>
       <c r="Y36" s="81" t="n">
         <v>1220</v>
@@ -7228,12 +7228,12 @@
         <f>SUM(AB37:AI37)</f>
         <v/>
       </c>
-      <c r="S37" s="81">
-        <f>AK37</f>
-        <v/>
-      </c>
-      <c r="T37" s="81" t="n">
-        <v>0</v>
+      <c r="S37" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" s="81">
+        <f>AM37</f>
+        <v/>
       </c>
       <c r="Y37" s="81" t="n">
         <v>1234</v>
@@ -7316,12 +7316,12 @@
         <f>SUM(AB38:AI38)</f>
         <v/>
       </c>
-      <c r="S38" s="85">
-        <f>AK38</f>
-        <v/>
-      </c>
-      <c r="T38" s="85" t="n">
-        <v>0</v>
+      <c r="S38" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" s="85">
+        <f>AM38</f>
+        <v/>
       </c>
       <c r="U38" s="86" t="n"/>
       <c r="V38" s="86" t="n"/>
@@ -7342,6 +7342,8 @@
       <c r="AI38" s="86" t="n"/>
       <c r="AJ38" s="86" t="n"/>
       <c r="AK38" s="86" t="n"/>
+      <c r="AL38" s="86" t="n"/>
+      <c r="AM38" s="86" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="72">
@@ -7413,12 +7415,12 @@
         <f>SUM(AB39:AI39)</f>
         <v/>
       </c>
-      <c r="S39" s="81">
-        <f>AK39</f>
-        <v/>
-      </c>
-      <c r="T39" s="81" t="n">
-        <v>0</v>
+      <c r="S39" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" s="81">
+        <f>AM39</f>
+        <v/>
       </c>
       <c r="Y39" s="81" t="n">
         <v>1230</v>
@@ -7506,12 +7508,12 @@
         <f>SUM(AB40:AI40)</f>
         <v/>
       </c>
-      <c r="S40" s="81">
-        <f>AK40</f>
-        <v/>
-      </c>
-      <c r="T40" s="81" t="n">
-        <v>0</v>
+      <c r="S40" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" s="81">
+        <f>AM40</f>
+        <v/>
       </c>
       <c r="Y40" s="81" t="n">
         <v>1249</v>
@@ -7531,7 +7533,7 @@
       <c r="AG40" s="81" t="n">
         <v>65</v>
       </c>
-      <c r="AK40" s="81" t="n">
+      <c r="AM40" s="81" t="n">
         <v>-374.7</v>
       </c>
     </row>
@@ -7602,12 +7604,12 @@
         <f>SUM(AB41:AI41)</f>
         <v/>
       </c>
-      <c r="S41" s="81">
-        <f>AK41</f>
-        <v/>
-      </c>
-      <c r="T41" s="81" t="n">
-        <v>0</v>
+      <c r="S41" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T41" s="81">
+        <f>AM41</f>
+        <v/>
       </c>
       <c r="Y41" s="81" t="n">
         <v>1325</v>
@@ -7693,12 +7695,12 @@
         <f>SUM(AB42:AI42)</f>
         <v/>
       </c>
-      <c r="S42" s="85">
-        <f>AK42</f>
-        <v/>
-      </c>
-      <c r="T42" s="85" t="n">
-        <v>0</v>
+      <c r="S42" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T42" s="85">
+        <f>AM42</f>
+        <v/>
       </c>
       <c r="U42" s="86" t="n"/>
       <c r="V42" s="86" t="n"/>
@@ -7719,6 +7721,8 @@
       <c r="AI42" s="86" t="n"/>
       <c r="AJ42" s="86" t="n"/>
       <c r="AK42" s="86" t="n"/>
+      <c r="AL42" s="86" t="n"/>
+      <c r="AM42" s="86" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="72">
@@ -7787,12 +7791,12 @@
         <f>SUM(AB43:AI43)</f>
         <v/>
       </c>
-      <c r="S43" s="81">
-        <f>AK43</f>
-        <v/>
-      </c>
-      <c r="T43" s="81" t="n">
-        <v>0</v>
+      <c r="S43" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" s="81">
+        <f>AM43</f>
+        <v/>
       </c>
       <c r="Y43" s="81" t="n">
         <v>1799</v>
@@ -7875,12 +7879,12 @@
         <f>SUM(AB44:AI44)</f>
         <v/>
       </c>
-      <c r="S44" s="85">
-        <f>AK44</f>
-        <v/>
-      </c>
-      <c r="T44" s="85" t="n">
-        <v>0</v>
+      <c r="S44" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" s="85">
+        <f>AM44</f>
+        <v/>
       </c>
       <c r="U44" s="86" t="n"/>
       <c r="V44" s="86" t="n"/>
@@ -7901,6 +7905,8 @@
       <c r="AI44" s="86" t="n"/>
       <c r="AJ44" s="86" t="n"/>
       <c r="AK44" s="86" t="n"/>
+      <c r="AL44" s="86" t="n"/>
+      <c r="AM44" s="86" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="83">
@@ -7964,12 +7970,12 @@
         <f>SUM(AB45:AI45)</f>
         <v/>
       </c>
-      <c r="S45" s="85">
-        <f>AK45</f>
-        <v/>
-      </c>
-      <c r="T45" s="85" t="n">
-        <v>0</v>
+      <c r="S45" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" s="85">
+        <f>AM45</f>
+        <v/>
       </c>
       <c r="U45" s="86" t="n"/>
       <c r="V45" s="86" t="n"/>
@@ -7990,6 +7996,8 @@
       <c r="AI45" s="86" t="n"/>
       <c r="AJ45" s="86" t="n"/>
       <c r="AK45" s="86" t="n"/>
+      <c r="AL45" s="86" t="n"/>
+      <c r="AM45" s="86" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="72">
@@ -8058,12 +8066,12 @@
         <f>SUM(AB46:AI46)</f>
         <v/>
       </c>
-      <c r="S46" s="81">
-        <f>AK46</f>
-        <v/>
-      </c>
-      <c r="T46" s="81" t="n">
-        <v>0</v>
+      <c r="S46" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" s="81">
+        <f>AM46</f>
+        <v/>
       </c>
       <c r="Y46" s="81" t="n">
         <v>1249</v>
@@ -8151,12 +8159,12 @@
         <f>SUM(AB47:AI47)</f>
         <v/>
       </c>
-      <c r="S47" s="81">
-        <f>AK47</f>
-        <v/>
-      </c>
-      <c r="T47" s="81" t="n">
-        <v>0</v>
+      <c r="S47" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T47" s="81">
+        <f>AM47</f>
+        <v/>
       </c>
       <c r="Y47" s="81" t="n">
         <v>1249</v>
@@ -8244,12 +8252,12 @@
         <f>SUM(AB48:AI48)</f>
         <v/>
       </c>
-      <c r="S48" s="81">
-        <f>AK48</f>
-        <v/>
-      </c>
-      <c r="T48" s="81" t="n">
-        <v>0</v>
+      <c r="S48" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T48" s="81">
+        <f>AM48</f>
+        <v/>
       </c>
       <c r="Y48" s="81" t="n">
         <v>1245</v>
@@ -8337,12 +8345,12 @@
         <f>SUM(AB49:AI49)</f>
         <v/>
       </c>
-      <c r="S49" s="81">
-        <f>AK49</f>
-        <v/>
-      </c>
-      <c r="T49" s="81" t="n">
-        <v>0</v>
+      <c r="S49" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" s="81">
+        <f>AM49</f>
+        <v/>
       </c>
       <c r="Y49" s="81" t="n">
         <v>1215</v>
@@ -8436,12 +8444,12 @@
         <f>SUM(AB50:AI50)</f>
         <v/>
       </c>
-      <c r="S50" s="81">
-        <f>AK50</f>
-        <v/>
-      </c>
-      <c r="T50" s="81" t="n">
-        <v>0</v>
+      <c r="S50" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T50" s="81">
+        <f>AM50</f>
+        <v/>
       </c>
       <c r="Y50" s="81" t="n">
         <v>1345</v>
@@ -8532,12 +8540,12 @@
         <f>SUM(AB51:AI51)</f>
         <v/>
       </c>
-      <c r="S51" s="81">
-        <f>AK51</f>
-        <v/>
-      </c>
-      <c r="T51" s="81" t="n">
-        <v>0</v>
+      <c r="S51" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T51" s="81">
+        <f>AM51</f>
+        <v/>
       </c>
       <c r="Y51" s="81" t="n">
         <v>1244</v>
@@ -8625,12 +8633,12 @@
         <f>SUM(AB52:AI52)</f>
         <v/>
       </c>
-      <c r="S52" s="81">
-        <f>AK52</f>
-        <v/>
-      </c>
-      <c r="T52" s="81" t="n">
-        <v>0</v>
+      <c r="S52" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T52" s="81">
+        <f>AM52</f>
+        <v/>
       </c>
       <c r="Y52" s="81" t="n">
         <v>1320</v>
@@ -8721,12 +8729,12 @@
         <f>SUM(AB53:AI53)</f>
         <v/>
       </c>
-      <c r="S53" s="81">
-        <f>AK53</f>
-        <v/>
-      </c>
-      <c r="T53" s="81" t="n">
-        <v>0</v>
+      <c r="S53" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T53" s="81">
+        <f>AM53</f>
+        <v/>
       </c>
       <c r="Y53" s="81" t="n">
         <v>1049</v>
@@ -8809,12 +8817,12 @@
         <f>SUM(AB54:AI54)</f>
         <v/>
       </c>
-      <c r="S54" s="85">
-        <f>AK54</f>
-        <v/>
-      </c>
-      <c r="T54" s="85" t="n">
-        <v>0</v>
+      <c r="S54" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T54" s="85">
+        <f>AM54</f>
+        <v/>
       </c>
       <c r="U54" s="86" t="n"/>
       <c r="V54" s="86" t="n"/>
@@ -8835,6 +8843,8 @@
       <c r="AI54" s="86" t="n"/>
       <c r="AJ54" s="86" t="n"/>
       <c r="AK54" s="86" t="n"/>
+      <c r="AL54" s="86" t="n"/>
+      <c r="AM54" s="86" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="83">
@@ -8898,12 +8908,12 @@
         <f>SUM(AB55:AI55)</f>
         <v/>
       </c>
-      <c r="S55" s="85">
-        <f>AK55</f>
-        <v/>
-      </c>
-      <c r="T55" s="85" t="n">
-        <v>0</v>
+      <c r="S55" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T55" s="85">
+        <f>AM55</f>
+        <v/>
       </c>
       <c r="U55" s="86" t="n"/>
       <c r="V55" s="86" t="n"/>
@@ -8924,6 +8934,8 @@
       <c r="AI55" s="86" t="n"/>
       <c r="AJ55" s="86" t="n"/>
       <c r="AK55" s="86" t="n"/>
+      <c r="AL55" s="86" t="n"/>
+      <c r="AM55" s="86" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="83">
@@ -8987,12 +8999,12 @@
         <f>SUM(AB56:AI56)</f>
         <v/>
       </c>
-      <c r="S56" s="85">
-        <f>AK56</f>
-        <v/>
-      </c>
-      <c r="T56" s="85" t="n">
-        <v>0</v>
+      <c r="S56" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T56" s="85">
+        <f>AM56</f>
+        <v/>
       </c>
       <c r="U56" s="86" t="n"/>
       <c r="V56" s="86" t="n"/>
@@ -9013,6 +9025,8 @@
       <c r="AI56" s="86" t="n"/>
       <c r="AJ56" s="86" t="n"/>
       <c r="AK56" s="86" t="n"/>
+      <c r="AL56" s="86" t="n"/>
+      <c r="AM56" s="86" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="72">
@@ -9081,12 +9095,12 @@
         <f>SUM(AB57:AI57)</f>
         <v/>
       </c>
-      <c r="S57" s="81">
-        <f>AK57</f>
-        <v/>
-      </c>
-      <c r="T57" s="81" t="n">
-        <v>0</v>
+      <c r="S57" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T57" s="81">
+        <f>AM57</f>
+        <v/>
       </c>
       <c r="Y57" s="81" t="n">
         <v>1139</v>
@@ -9174,12 +9188,12 @@
         <f>SUM(AB58:AI58)</f>
         <v/>
       </c>
-      <c r="S58" s="81">
-        <f>AK58</f>
-        <v/>
-      </c>
-      <c r="T58" s="81" t="n">
-        <v>0</v>
+      <c r="S58" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T58" s="81">
+        <f>AM58</f>
+        <v/>
       </c>
       <c r="Y58" s="81" t="n">
         <v>1099</v>
@@ -9264,12 +9278,12 @@
         <f>SUM(AB59:AI59)</f>
         <v/>
       </c>
-      <c r="S59" s="81">
-        <f>AK59</f>
-        <v/>
-      </c>
-      <c r="T59" s="81" t="n">
-        <v>0</v>
+      <c r="S59" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T59" s="81">
+        <f>AM59</f>
+        <v/>
       </c>
       <c r="Y59" s="81" t="n">
         <v>990</v>
@@ -9360,12 +9374,12 @@
         <f>SUM(AB60:AI60)</f>
         <v/>
       </c>
-      <c r="S60" s="81">
-        <f>AK60</f>
-        <v/>
-      </c>
-      <c r="T60" s="81" t="n">
-        <v>0</v>
+      <c r="S60" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T60" s="81">
+        <f>AM60</f>
+        <v/>
       </c>
       <c r="Y60" s="81" t="n">
         <v>1125</v>
@@ -9453,12 +9467,12 @@
         <f>SUM(AB61:AI61)</f>
         <v/>
       </c>
-      <c r="S61" s="81">
-        <f>AK61</f>
-        <v/>
-      </c>
-      <c r="T61" s="81" t="n">
-        <v>0</v>
+      <c r="S61" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T61" s="81">
+        <f>AM61</f>
+        <v/>
       </c>
       <c r="Y61" s="81" t="n">
         <v>1179</v>
@@ -9546,12 +9560,12 @@
         <f>SUM(AB62:AI62)</f>
         <v/>
       </c>
-      <c r="S62" s="81">
-        <f>AK62</f>
-        <v/>
-      </c>
-      <c r="T62" s="81" t="n">
-        <v>0</v>
+      <c r="S62" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T62" s="81">
+        <f>AM62</f>
+        <v/>
       </c>
       <c r="Y62" s="81" t="n">
         <v>1124</v>
@@ -9639,12 +9653,12 @@
         <f>SUM(AB63:AI63)</f>
         <v/>
       </c>
-      <c r="S63" s="81">
-        <f>AK63</f>
-        <v/>
-      </c>
-      <c r="T63" s="81" t="n">
-        <v>0</v>
+      <c r="S63" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T63" s="81">
+        <f>AM63</f>
+        <v/>
       </c>
       <c r="Y63" s="81" t="n">
         <v>1324</v>
@@ -9735,12 +9749,12 @@
         <f>SUM(AB64:AI64)</f>
         <v/>
       </c>
-      <c r="S64" s="81">
-        <f>AK64</f>
-        <v/>
-      </c>
-      <c r="T64" s="81" t="n">
-        <v>0</v>
+      <c r="S64" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T64" s="81">
+        <f>AM64</f>
+        <v/>
       </c>
       <c r="Y64" s="81" t="n">
         <v>1114</v>
@@ -9828,12 +9842,12 @@
         <f>SUM(AB65:AI65)</f>
         <v/>
       </c>
-      <c r="S65" s="81">
-        <f>AK65</f>
-        <v/>
-      </c>
-      <c r="T65" s="81" t="n">
-        <v>0</v>
+      <c r="S65" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T65" s="81">
+        <f>AM65</f>
+        <v/>
       </c>
       <c r="Y65" s="81" t="n">
         <v>1245</v>
@@ -9921,12 +9935,12 @@
         <f>SUM(AB66:AI66)</f>
         <v/>
       </c>
-      <c r="S66" s="81">
-        <f>AK66</f>
-        <v/>
-      </c>
-      <c r="T66" s="81" t="n">
-        <v>0</v>
+      <c r="S66" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T66" s="81">
+        <f>AM66</f>
+        <v/>
       </c>
       <c r="Y66" s="81" t="n">
         <v>1059</v>
@@ -10014,12 +10028,12 @@
         <f>SUM(AB67:AI67)</f>
         <v/>
       </c>
-      <c r="S67" s="81">
-        <f>AK67</f>
-        <v/>
-      </c>
-      <c r="T67" s="81" t="n">
-        <v>0</v>
+      <c r="S67" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T67" s="81">
+        <f>AM67</f>
+        <v/>
       </c>
       <c r="Y67" s="81" t="n">
         <v>1384</v>
@@ -10102,12 +10116,12 @@
         <f>SUM(AB68:AI68)</f>
         <v/>
       </c>
-      <c r="S68" s="85">
-        <f>AK68</f>
-        <v/>
-      </c>
-      <c r="T68" s="85" t="n">
-        <v>0</v>
+      <c r="S68" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T68" s="85">
+        <f>AM68</f>
+        <v/>
       </c>
       <c r="U68" s="86" t="n"/>
       <c r="V68" s="86" t="n"/>
@@ -10128,6 +10142,8 @@
       <c r="AI68" s="86" t="n"/>
       <c r="AJ68" s="86" t="n"/>
       <c r="AK68" s="86" t="n"/>
+      <c r="AL68" s="86" t="n"/>
+      <c r="AM68" s="86" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="72">
@@ -10196,12 +10212,12 @@
         <f>SUM(AB69:AI69)</f>
         <v/>
       </c>
-      <c r="S69" s="81">
-        <f>AK69</f>
-        <v/>
-      </c>
-      <c r="T69" s="81" t="n">
-        <v>0</v>
+      <c r="S69" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T69" s="81">
+        <f>AM69</f>
+        <v/>
       </c>
       <c r="Y69" s="81" t="n">
         <v>1184</v>
@@ -10292,12 +10308,12 @@
         <f>SUM(AB70:AI70)</f>
         <v/>
       </c>
-      <c r="S70" s="81">
-        <f>AK70</f>
-        <v/>
-      </c>
-      <c r="T70" s="81" t="n">
-        <v>0</v>
+      <c r="S70" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T70" s="81">
+        <f>AM70</f>
+        <v/>
       </c>
       <c r="Y70" s="81" t="n">
         <v>1255</v>
@@ -10385,12 +10401,12 @@
         <f>SUM(AB71:AI71)</f>
         <v/>
       </c>
-      <c r="S71" s="81">
-        <f>AK71</f>
-        <v/>
-      </c>
-      <c r="T71" s="81" t="n">
-        <v>0</v>
+      <c r="S71" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T71" s="81">
+        <f>AM71</f>
+        <v/>
       </c>
       <c r="Y71" s="81" t="n">
         <v>1149</v>
@@ -10473,12 +10489,12 @@
         <f>SUM(AB72:AI72)</f>
         <v/>
       </c>
-      <c r="S72" s="85">
-        <f>AK72</f>
-        <v/>
-      </c>
-      <c r="T72" s="85" t="n">
-        <v>0</v>
+      <c r="S72" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="T72" s="85">
+        <f>AM72</f>
+        <v/>
       </c>
       <c r="U72" s="86" t="n"/>
       <c r="V72" s="86" t="n"/>
@@ -10499,6 +10515,8 @@
       <c r="AI72" s="86" t="n"/>
       <c r="AJ72" s="86" t="n"/>
       <c r="AK72" s="86" t="n"/>
+      <c r="AL72" s="86" t="n"/>
+      <c r="AM72" s="86" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="72">
@@ -10567,12 +10585,12 @@
         <f>SUM(AB73:AI73)</f>
         <v/>
       </c>
-      <c r="S73" s="81">
-        <f>AK73</f>
-        <v/>
-      </c>
-      <c r="T73" s="81" t="n">
-        <v>0</v>
+      <c r="S73" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T73" s="81">
+        <f>AM73</f>
+        <v/>
       </c>
       <c r="Y73" s="81" t="n">
         <v>1330</v>
@@ -10660,12 +10678,12 @@
         <f>SUM(AB74:AI74)</f>
         <v/>
       </c>
-      <c r="S74" s="81">
-        <f>AK74</f>
-        <v/>
-      </c>
-      <c r="T74" s="81" t="n">
-        <v>0</v>
+      <c r="S74" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T74" s="81">
+        <f>AM74</f>
+        <v/>
       </c>
       <c r="Y74" s="81" t="n">
         <v>1185</v>
@@ -10756,12 +10774,12 @@
         <f>SUM(AB75:AI75)</f>
         <v/>
       </c>
-      <c r="S75" s="81">
-        <f>AK75</f>
-        <v/>
-      </c>
-      <c r="T75" s="81" t="n">
-        <v>0</v>
+      <c r="S75" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T75" s="81">
+        <f>AM75</f>
+        <v/>
       </c>
       <c r="Y75" s="81" t="n">
         <v>1355</v>
@@ -10852,12 +10870,12 @@
         <f>SUM(AB76:AI76)</f>
         <v/>
       </c>
-      <c r="S76" s="81">
-        <f>AK76</f>
-        <v/>
-      </c>
-      <c r="T76" s="81" t="n">
-        <v>0</v>
+      <c r="S76" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T76" s="81">
+        <f>AM76</f>
+        <v/>
       </c>
       <c r="Y76" s="81" t="n">
         <v>1334</v>
@@ -10945,12 +10963,12 @@
         <f>SUM(AB77:AI77)</f>
         <v/>
       </c>
-      <c r="S77" s="81">
-        <f>AK77</f>
-        <v/>
-      </c>
-      <c r="T77" s="81" t="n">
-        <v>0</v>
+      <c r="S77" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T77" s="81">
+        <f>AM77</f>
+        <v/>
       </c>
       <c r="Y77" s="81" t="n">
         <v>1124</v>
@@ -11038,12 +11056,12 @@
         <f>SUM(AB78:AI78)</f>
         <v/>
       </c>
-      <c r="S78" s="81">
-        <f>AK78</f>
-        <v/>
-      </c>
-      <c r="T78" s="81" t="n">
-        <v>0</v>
+      <c r="S78" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T78" s="81">
+        <f>AM78</f>
+        <v/>
       </c>
       <c r="Y78" s="81" t="n">
         <v>1334</v>
@@ -11131,12 +11149,12 @@
         <f>SUM(AB79:AI79)</f>
         <v/>
       </c>
-      <c r="S79" s="81">
-        <f>AK79</f>
-        <v/>
-      </c>
-      <c r="T79" s="81" t="n">
-        <v>0</v>
+      <c r="S79" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T79" s="81">
+        <f>AM79</f>
+        <v/>
       </c>
       <c r="Y79" s="81" t="n">
         <v>1394</v>
@@ -11224,12 +11242,12 @@
         <f>SUM(AB80:AI80)</f>
         <v/>
       </c>
-      <c r="S80" s="81">
-        <f>AK80</f>
-        <v/>
-      </c>
-      <c r="T80" s="81" t="n">
-        <v>0</v>
+      <c r="S80" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T80" s="81">
+        <f>AM80</f>
+        <v/>
       </c>
       <c r="Y80" s="81" t="n">
         <v>1300</v>
@@ -11320,12 +11338,12 @@
         <f>SUM(AB81:AI81)</f>
         <v/>
       </c>
-      <c r="S81" s="81">
-        <f>AK81</f>
-        <v/>
-      </c>
-      <c r="T81" s="81" t="n">
-        <v>0</v>
+      <c r="S81" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T81" s="81">
+        <f>AM81</f>
+        <v/>
       </c>
       <c r="Y81" s="81" t="n">
         <v>1145</v>
@@ -11419,12 +11437,12 @@
         <f>SUM(AB82:AI82)</f>
         <v/>
       </c>
-      <c r="S82" s="81">
-        <f>AK82</f>
-        <v/>
-      </c>
-      <c r="T82" s="81" t="n">
-        <v>0</v>
+      <c r="S82" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T82" s="81">
+        <f>AM82</f>
+        <v/>
       </c>
       <c r="Y82" s="81" t="n">
         <v>1189</v>

</xml_diff>

<commit_message>
OneLineRR: place pet-related Other Income charges leftmost
In the Other Income section, any line item whose name contains "pet" is moved
to the leftmost column(s); remaining items keep their first-seen order.

Maven: "Pet Rent" is now the first Other Income column (AB). Heritage passes.
Docs + iteration log (#24) updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Birgo RR Exhibits - Maven @ 806v07.01.26.xlsx
+++ b/examples/outputs/Birgo RR Exhibits - Maven @ 806v07.01.26.xlsx
@@ -6647,12 +6647,12 @@
       </c>
       <c r="AB31" s="67" t="inlineStr">
         <is>
+          <t>Pet Rent</t>
+        </is>
+      </c>
+      <c r="AC31" s="67" t="inlineStr">
+        <is>
           <t>Building Protection Policy</t>
-        </is>
-      </c>
-      <c r="AC31" s="67" t="inlineStr">
-        <is>
-          <t>Pet Rent</t>
         </is>
       </c>
       <c r="AD31" s="67" t="inlineStr">
@@ -6768,10 +6768,10 @@
         <v>1285</v>
       </c>
       <c r="AB32" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC32" s="81" t="n">
         <v>15</v>
-      </c>
-      <c r="AC32" s="81" t="n">
-        <v>35</v>
       </c>
       <c r="AD32" s="81" t="n">
         <v>5</v>
@@ -6866,7 +6866,7 @@
       <c r="Y33" s="81" t="n">
         <v>1229</v>
       </c>
-      <c r="AB33" s="81" t="n">
+      <c r="AC33" s="81" t="n">
         <v>12</v>
       </c>
       <c r="AD33" s="81" t="n">
@@ -6959,7 +6959,7 @@
       <c r="Y34" s="81" t="n">
         <v>1249</v>
       </c>
-      <c r="AB34" s="81" t="n">
+      <c r="AC34" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD34" s="81" t="n">
@@ -7052,7 +7052,7 @@
       <c r="Y35" s="81" t="n">
         <v>1239</v>
       </c>
-      <c r="AB35" s="81" t="n">
+      <c r="AC35" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD35" s="81" t="n">
@@ -7145,7 +7145,7 @@
       <c r="Y36" s="81" t="n">
         <v>1220</v>
       </c>
-      <c r="AB36" s="81" t="n">
+      <c r="AC36" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD36" s="81" t="n">
@@ -7238,7 +7238,7 @@
       <c r="Y37" s="81" t="n">
         <v>1234</v>
       </c>
-      <c r="AB37" s="81" t="n">
+      <c r="AC37" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD37" s="81" t="n">
@@ -7425,7 +7425,7 @@
       <c r="Y39" s="81" t="n">
         <v>1230</v>
       </c>
-      <c r="AB39" s="81" t="n">
+      <c r="AC39" s="81" t="n">
         <v>12</v>
       </c>
       <c r="AD39" s="81" t="n">
@@ -7518,7 +7518,7 @@
       <c r="Y40" s="81" t="n">
         <v>1249</v>
       </c>
-      <c r="AB40" s="81" t="n">
+      <c r="AC40" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD40" s="81" t="n">
@@ -7615,10 +7615,10 @@
         <v>1325</v>
       </c>
       <c r="AB41" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC41" s="81" t="n">
         <v>12</v>
-      </c>
-      <c r="AC41" s="81" t="n">
-        <v>35</v>
       </c>
       <c r="AD41" s="81" t="n">
         <v>5</v>
@@ -7801,7 +7801,7 @@
       <c r="Y43" s="81" t="n">
         <v>1799</v>
       </c>
-      <c r="AB43" s="81" t="n">
+      <c r="AC43" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD43" s="81" t="n">
@@ -8076,7 +8076,7 @@
       <c r="Y46" s="81" t="n">
         <v>1249</v>
       </c>
-      <c r="AB46" s="81" t="n">
+      <c r="AC46" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD46" s="81" t="n">
@@ -8169,7 +8169,7 @@
       <c r="Y47" s="81" t="n">
         <v>1249</v>
       </c>
-      <c r="AB47" s="81" t="n">
+      <c r="AC47" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD47" s="81" t="n">
@@ -8262,7 +8262,7 @@
       <c r="Y48" s="81" t="n">
         <v>1245</v>
       </c>
-      <c r="AB48" s="81" t="n">
+      <c r="AC48" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD48" s="81" t="n">
@@ -8356,10 +8356,10 @@
         <v>1215</v>
       </c>
       <c r="AB49" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="AC49" s="81" t="n">
         <v>12</v>
-      </c>
-      <c r="AC49" s="81" t="n">
-        <v>30</v>
       </c>
       <c r="AD49" s="81" t="n">
         <v>5</v>
@@ -8455,10 +8455,10 @@
         <v>1345</v>
       </c>
       <c r="AB50" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC50" s="81" t="n">
         <v>12</v>
-      </c>
-      <c r="AC50" s="81" t="n">
-        <v>35</v>
       </c>
       <c r="AD50" s="81" t="n">
         <v>5</v>
@@ -8550,7 +8550,7 @@
       <c r="Y51" s="81" t="n">
         <v>1244</v>
       </c>
-      <c r="AB51" s="81" t="n">
+      <c r="AC51" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD51" s="81" t="n">
@@ -8644,10 +8644,10 @@
         <v>1320</v>
       </c>
       <c r="AB52" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC52" s="81" t="n">
         <v>12</v>
-      </c>
-      <c r="AC52" s="81" t="n">
-        <v>35</v>
       </c>
       <c r="AD52" s="81" t="n">
         <v>5</v>
@@ -8739,7 +8739,7 @@
       <c r="Y53" s="81" t="n">
         <v>1049</v>
       </c>
-      <c r="AB53" s="81" t="n">
+      <c r="AC53" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD53" s="81" t="n">
@@ -9105,7 +9105,7 @@
       <c r="Y57" s="81" t="n">
         <v>1139</v>
       </c>
-      <c r="AB57" s="81" t="n">
+      <c r="AC57" s="81" t="n">
         <v>12</v>
       </c>
       <c r="AD57" s="81" t="n">
@@ -9198,7 +9198,7 @@
       <c r="Y58" s="81" t="n">
         <v>1099</v>
       </c>
-      <c r="AB58" s="81" t="n">
+      <c r="AC58" s="81" t="n">
         <v>12</v>
       </c>
       <c r="AD58" s="81" t="n">
@@ -9288,7 +9288,7 @@
       <c r="Y59" s="81" t="n">
         <v>990</v>
       </c>
-      <c r="AB59" s="81" t="n">
+      <c r="AC59" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD59" s="81" t="n">
@@ -9384,7 +9384,7 @@
       <c r="Y60" s="81" t="n">
         <v>1125</v>
       </c>
-      <c r="AB60" s="81" t="n">
+      <c r="AC60" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD60" s="81" t="n">
@@ -9477,7 +9477,7 @@
       <c r="Y61" s="81" t="n">
         <v>1179</v>
       </c>
-      <c r="AB61" s="81" t="n">
+      <c r="AC61" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD61" s="81" t="n">
@@ -9570,7 +9570,7 @@
       <c r="Y62" s="81" t="n">
         <v>1124</v>
       </c>
-      <c r="AB62" s="81" t="n">
+      <c r="AC62" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD62" s="81" t="n">
@@ -9664,10 +9664,10 @@
         <v>1324</v>
       </c>
       <c r="AB63" s="81" t="n">
+        <v>30</v>
+      </c>
+      <c r="AC63" s="81" t="n">
         <v>15</v>
-      </c>
-      <c r="AC63" s="81" t="n">
-        <v>30</v>
       </c>
       <c r="AD63" s="81" t="n">
         <v>5</v>
@@ -9759,7 +9759,7 @@
       <c r="Y64" s="81" t="n">
         <v>1114</v>
       </c>
-      <c r="AB64" s="81" t="n">
+      <c r="AC64" s="81" t="n">
         <v>12</v>
       </c>
       <c r="AD64" s="81" t="n">
@@ -9852,7 +9852,7 @@
       <c r="Y65" s="81" t="n">
         <v>1245</v>
       </c>
-      <c r="AB65" s="81" t="n">
+      <c r="AC65" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD65" s="81" t="n">
@@ -9945,7 +9945,7 @@
       <c r="Y66" s="81" t="n">
         <v>1059</v>
       </c>
-      <c r="AB66" s="81" t="n">
+      <c r="AC66" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD66" s="81" t="n">
@@ -10038,7 +10038,7 @@
       <c r="Y67" s="81" t="n">
         <v>1384</v>
       </c>
-      <c r="AB67" s="81" t="n">
+      <c r="AC67" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD67" s="81" t="n">
@@ -10223,10 +10223,10 @@
         <v>1184</v>
       </c>
       <c r="AB69" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC69" s="81" t="n">
         <v>15</v>
-      </c>
-      <c r="AC69" s="81" t="n">
-        <v>35</v>
       </c>
       <c r="AD69" s="81" t="n">
         <v>5</v>
@@ -10318,7 +10318,7 @@
       <c r="Y70" s="81" t="n">
         <v>1255</v>
       </c>
-      <c r="AB70" s="81" t="n">
+      <c r="AC70" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD70" s="81" t="n">
@@ -10411,7 +10411,7 @@
       <c r="Y71" s="81" t="n">
         <v>1149</v>
       </c>
-      <c r="AB71" s="81" t="n">
+      <c r="AC71" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD71" s="81" t="n">
@@ -10595,7 +10595,7 @@
       <c r="Y73" s="81" t="n">
         <v>1330</v>
       </c>
-      <c r="AB73" s="81" t="n">
+      <c r="AC73" s="81" t="n">
         <v>12</v>
       </c>
       <c r="AD73" s="81" t="n">
@@ -10689,10 +10689,10 @@
         <v>1185</v>
       </c>
       <c r="AB74" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC74" s="81" t="n">
         <v>12</v>
-      </c>
-      <c r="AC74" s="81" t="n">
-        <v>35</v>
       </c>
       <c r="AD74" s="81" t="n">
         <v>5</v>
@@ -10785,10 +10785,10 @@
         <v>1355</v>
       </c>
       <c r="AB75" s="81" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC75" s="81" t="n">
         <v>15</v>
-      </c>
-      <c r="AC75" s="81" t="n">
-        <v>35</v>
       </c>
       <c r="AD75" s="81" t="n">
         <v>5</v>
@@ -10880,7 +10880,7 @@
       <c r="Y76" s="81" t="n">
         <v>1334</v>
       </c>
-      <c r="AB76" s="81" t="n">
+      <c r="AC76" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD76" s="81" t="n">
@@ -10973,7 +10973,7 @@
       <c r="Y77" s="81" t="n">
         <v>1124</v>
       </c>
-      <c r="AB77" s="81" t="n">
+      <c r="AC77" s="81" t="n">
         <v>12</v>
       </c>
       <c r="AD77" s="81" t="n">
@@ -11066,7 +11066,7 @@
       <c r="Y78" s="81" t="n">
         <v>1334</v>
       </c>
-      <c r="AB78" s="81" t="n">
+      <c r="AC78" s="81" t="n">
         <v>12</v>
       </c>
       <c r="AD78" s="81" t="n">
@@ -11159,7 +11159,7 @@
       <c r="Y79" s="81" t="n">
         <v>1394</v>
       </c>
-      <c r="AB79" s="81" t="n">
+      <c r="AC79" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD79" s="81" t="n">
@@ -11252,7 +11252,7 @@
       <c r="Y80" s="81" t="n">
         <v>1300</v>
       </c>
-      <c r="AB80" s="81" t="n">
+      <c r="AC80" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD80" s="81" t="n">
@@ -11349,10 +11349,10 @@
         <v>1145</v>
       </c>
       <c r="AB81" s="81" t="n">
+        <v>65</v>
+      </c>
+      <c r="AC81" s="81" t="n">
         <v>12</v>
-      </c>
-      <c r="AC81" s="81" t="n">
-        <v>65</v>
       </c>
       <c r="AD81" s="81" t="n">
         <v>5</v>
@@ -11447,7 +11447,7 @@
       <c r="Y82" s="81" t="n">
         <v>1189</v>
       </c>
-      <c r="AB82" s="81" t="n">
+      <c r="AC82" s="81" t="n">
         <v>15</v>
       </c>
       <c r="AD82" s="81" t="n">

</xml_diff>